<commit_message>
ok test function register
</commit_message>
<xml_diff>
--- a/data/data_test.xlsx
+++ b/data/data_test.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnTotNghiep_NguyenQuyen_10122312\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC01716-D811-4C0B-B4EB-E3E4AA97C9A1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0C3480-E968-4B96-87B9-85712ACDF376}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8010" xr2:uid="{A15DE430-7E6B-4467-9607-107A07875CE8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8010" activeTab="1" xr2:uid="{A15DE430-7E6B-4467-9607-107A07875CE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="Search" sheetId="3" r:id="rId2"/>
+    <sheet name="Register" sheetId="4" r:id="rId2"/>
+    <sheet name="Search" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="41">
   <si>
     <t>tuyetmai99@gmail.com</t>
   </si>
@@ -89,6 +90,66 @@
   </si>
   <si>
     <t>Thoát</t>
+  </si>
+  <si>
+    <t>${re_password}</t>
+  </si>
+  <si>
+    <t>huyentrang@gmail</t>
+  </si>
+  <si>
+    <t>huyentrang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">huyentrang </t>
+  </si>
+  <si>
+    <t>huyentrang@gmail.com</t>
+  </si>
+  <si>
+    <t>Email không đúng định dạng</t>
+  </si>
+  <si>
+    <t>huyentrang@</t>
+  </si>
+  <si>
+    <t>@gmail</t>
+  </si>
+  <si>
+    <t>huyentrang@.com</t>
+  </si>
+  <si>
+    <t>huyen</t>
+  </si>
+  <si>
+    <t>Mật khẩu tối thiểu phải có 6 ký tự</t>
+  </si>
+  <si>
+    <t>Xác nhận mật khẩu không chính xác</t>
+  </si>
+  <si>
+    <t>abcdefg</t>
+  </si>
+  <si>
+    <t>invalid</t>
+  </si>
+  <si>
+    <t>Email đã được sử dụng</t>
+  </si>
+  <si>
+    <t>ducthuan@gmail.com</t>
+  </si>
+  <si>
+    <t>ducthuan</t>
+  </si>
+  <si>
+    <t>linhchi@gmail.vn</t>
+  </si>
+  <si>
+    <t>linhchi</t>
+  </si>
+  <si>
+    <t>linhchi@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -133,7 +194,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -141,6 +202,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -574,6 +638,201 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96B7BD28-F33A-4951-B834-32B5C346E3E5}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6328125" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" customWidth="1"/>
+    <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="4"/>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A12" r:id="rId1" xr:uid="{FB8CD489-1C7F-4608-8399-67E3A2B6F90E}"/>
+    <hyperlink ref="A13" r:id="rId2" xr:uid="{D9807A41-932E-4E66-A6EA-1F170A2C263A}"/>
+    <hyperlink ref="D13" r:id="rId3" xr:uid="{CDE2719E-E5C1-487F-A0D8-6581CBA38DFA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667F2FF2-D70E-4CEB-89DF-FD887F6CFB59}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>